<commit_message>
Update DF site info, output updated site info and eof dataset, including only Q and N related variables
</commit_message>
<xml_diff>
--- a/00_Data/Metadata/DiscoveryFarms_SiteLocations.xlsx
+++ b/00_Data/Metadata/DiscoveryFarms_SiteLocations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ealbright2\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwprod-my.sharepoint.com/personal/zchen2545_wisc_edu/Documents/Research/Discovery Farms/DF Runoff Generation/Github repo/DF_runoff/00_Data/Metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{204C13C8-A6DD-421F-BB9F-72257FF22DCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-7005" windowWidth="29040" windowHeight="15720" xr2:uid="{E5B6834D-12EE-4DD5-83BB-B14B22259238}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{E5B6834D-12EE-4DD5-83BB-B14B22259238}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -500,8 +500,8 @@
   </cellStyleXfs>
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">

</xml_diff>